<commit_message>
Updated temperature crosswalk file with Trinity water year for Trinity related temperatures
</commit_message>
<xml_diff>
--- a/inputs/location_code_crosswalk_Temp.xlsx
+++ b/inputs/location_code_crosswalk_Temp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emadonna\eis-appendix-generation\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\calsim_gits\eis-appendix-gen_upd\eis-appendix-generation\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8ED5ADAB-0330-4AB0-8E55-DC544538414F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C165D026-EEEF-454E-A562-FE2F219E7EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12135" yWindow="5835" windowWidth="17940" windowHeight="15060" xr2:uid="{0DD05B07-40C5-49AA-BF54-F3504D9FBA4C}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{0DD05B07-40C5-49AA-BF54-F3504D9FBA4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="121">
   <si>
     <t>Location (Title)</t>
   </si>
@@ -450,13 +450,16 @@
   </si>
   <si>
     <t>F.2.11-20</t>
+  </si>
+  <si>
+    <t>TRIN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -490,14 +493,8 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -513,6 +510,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00FF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -560,7 +563,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -602,6 +605,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -619,14 +628,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -664,7 +669,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -770,7 +775,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -912,7 +917,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -944,10 +949,17 @@
   <dimension ref="A1:P25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
+    <col min="3" max="3" width="58.42578125" customWidth="1"/>
+    <col min="4" max="4" width="40.42578125" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="20.5703125" customWidth="1"/>
+    <col min="7" max="7" width="22.42578125" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+    <col min="9" max="9" width="21" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -1007,7 +1019,7 @@
       <c r="B2" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="16" t="s">
         <v>14</v>
       </c>
       <c r="D2" s="4" t="s">
@@ -1029,8 +1041,8 @@
       <c r="J2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>21</v>
+      <c r="K2" s="15" t="s">
+        <v>120</v>
       </c>
       <c r="L2" s="6" t="b">
         <v>0</v>
@@ -1847,8 +1859,8 @@
       <c r="J19" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="K19" s="9" t="s">
-        <v>21</v>
+      <c r="K19" s="15" t="s">
+        <v>120</v>
       </c>
       <c r="L19" s="10" t="b">
         <v>0</v>
@@ -1895,8 +1907,8 @@
       <c r="J20" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="K20" s="9" t="s">
-        <v>21</v>
+      <c r="K20" s="15" t="s">
+        <v>120</v>
       </c>
       <c r="L20" s="10" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Fixed exceedance plot min/max values so the very highest and lowest %exceedance values aren't truncated
</commit_message>
<xml_diff>
--- a/inputs/location_code_crosswalk_Temp.xlsx
+++ b/inputs/location_code_crosswalk_Temp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\calsim_gits\eis-appendix-gen_upd\eis-appendix-generation\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C165D026-EEEF-454E-A562-FE2F219E7EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962172F1-1EA4-4BEB-9625-84CA4FD6A700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{0DD05B07-40C5-49AA-BF54-F3504D9FBA4C}"/>
+    <workbookView xWindow="-33570" yWindow="2685" windowWidth="32760" windowHeight="12960" xr2:uid="{0DD05B07-40C5-49AA-BF54-F3504D9FBA4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="126">
   <si>
     <t>Location (Title)</t>
   </si>
@@ -453,6 +453,21 @@
   </si>
   <si>
     <t>TRIN</t>
+  </si>
+  <si>
+    <t>Below Trinity</t>
+  </si>
+  <si>
+    <t>Above Lewiston</t>
+  </si>
+  <si>
+    <t>Below Lewiston</t>
+  </si>
+  <si>
+    <t>Douglas City</t>
+  </si>
+  <si>
+    <t>North Fork Trinity</t>
   </si>
 </sst>
 </file>
@@ -494,7 +509,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -516,6 +531,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -563,7 +584,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -609,6 +630,19 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -946,7 +980,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09E1BEF8-AB6B-4CC1-898E-F8639CC22C68}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" customWidth="1"/>
@@ -955,7 +989,7 @@
     <col min="4" max="4" width="40.42578125" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="20.5703125" customWidth="1"/>
-    <col min="7" max="7" width="22.42578125" customWidth="1"/>
+    <col min="7" max="7" width="42.7109375" customWidth="1"/>
     <col min="8" max="8" width="28" customWidth="1"/>
     <col min="9" max="9" width="21" customWidth="1"/>
     <col min="10" max="10" width="18.85546875" customWidth="1"/>
@@ -2161,6 +2195,226 @@
         <v>80</v>
       </c>
     </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="I26" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="J26" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="K26" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="L26" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M26" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="N26" s="17">
+        <v>2</v>
+      </c>
+      <c r="O26" s="21">
+        <v>42</v>
+      </c>
+      <c r="P26" s="21">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="I27" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="J27" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="L27" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M27" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="N27" s="17">
+        <v>2</v>
+      </c>
+      <c r="O27" s="21">
+        <v>42</v>
+      </c>
+      <c r="P27" s="21">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="J28" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="K28" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="L28" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M28" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="N28" s="17">
+        <v>2</v>
+      </c>
+      <c r="O28" s="21">
+        <v>42</v>
+      </c>
+      <c r="P28" s="21">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="I29" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="J29" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="K29" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="L29" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M29" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="N29" s="17">
+        <v>2</v>
+      </c>
+      <c r="O29" s="21">
+        <v>42</v>
+      </c>
+      <c r="P29" s="21">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C30" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="I30" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="J30" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="K30" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="L30" s="20" t="b">
+        <v>0</v>
+      </c>
+      <c r="M30" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="N30" s="17">
+        <v>2</v>
+      </c>
+      <c r="O30" s="21">
+        <v>42</v>
+      </c>
+      <c r="P30" s="21">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>